<commit_message>
Fix specs, add 0023_core
</commit_message>
<xml_diff>
--- a/Issues_No_Tests_final.xlsx
+++ b/Issues_No_Tests_final.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P89"/>
+  <dimension ref="A1:U89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -444,6 +444,11 @@
     <col width="55" customWidth="1" min="14" max="14"/>
     <col width="16" customWidth="1" min="15" max="15"/>
     <col width="40" customWidth="1" min="16" max="16"/>
+    <col width="34" customWidth="1" min="17" max="17"/>
+    <col width="20" customWidth="1" min="18" max="18"/>
+    <col width="20" customWidth="1" min="19" max="19"/>
+    <col width="18" customWidth="1" min="20" max="20"/>
+    <col width="20" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -527,6 +532,31 @@
           <t>Manual Review Note</t>
         </is>
       </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Domain</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>Composition</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>Science Difficulty</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>SWE Difficulty</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>science_relevance</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="B2" t="inlineStr">
@@ -590,6 +620,31 @@
           <t>Pass</t>
         </is>
       </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>Materials Science</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>joint</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>sufficient</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="B3" t="inlineStr">
@@ -654,6 +709,31 @@
           <t>Pass</t>
         </is>
       </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>Physics</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>joint</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>sufficient</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="B4" t="inlineStr">
@@ -717,6 +797,31 @@
           <t>Pass</t>
         </is>
       </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>Physics</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>joint</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>sufficient</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="B5" t="inlineStr">
@@ -780,6 +885,31 @@
           <t>Pass</t>
         </is>
       </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>Materials Science</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>joint</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>sufficient</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="B6" t="inlineStr">
@@ -843,6 +973,31 @@
           <t>Pass</t>
         </is>
       </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>Materials Science</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>swe_dominant</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>sufficient</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="B7" t="inlineStr">
@@ -906,6 +1061,31 @@
           <t>Pass</t>
         </is>
       </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>Materials Science</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>swe_dominant</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>sufficient</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="B8" t="inlineStr">
@@ -969,6 +1149,31 @@
           <t>Pass</t>
         </is>
       </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>Materials Science</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>joint</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>sufficient</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="B9" t="inlineStr">
@@ -1032,6 +1237,31 @@
           <t>Pass</t>
         </is>
       </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>Physics</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>joint</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>sufficient</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="B10" t="inlineStr">
@@ -1095,6 +1325,31 @@
           <t>Update: only keep issue 4180</t>
         </is>
       </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>Physics</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>joint</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>sufficient</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="B11" t="inlineStr">
@@ -1158,6 +1413,31 @@
           <t>Pass: gpt fail due to model quality / randomness</t>
         </is>
       </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>Materials Science</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>joint</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>sufficient</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="B12" t="inlineStr">
@@ -1221,6 +1501,31 @@
           <t>Pass</t>
         </is>
       </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>Chemistry</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>joint</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>sufficient</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="B13" t="inlineStr">
@@ -1284,6 +1589,31 @@
           <t>Update: add another two PR-paired issues https://github.com/lammps/lammps/issues/4337 and https://github.com/lammps/lammps/issues/4216</t>
         </is>
       </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>Materials Science</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>swe_dominant</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>sufficient</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="B14" t="inlineStr">
@@ -1347,6 +1677,31 @@
           <t>Update: add another two PR-paired issues https://github.com/lammps/lammps/issues/4337 and https://github.com/lammps/lammps/issues/4216</t>
         </is>
       </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>Materials Science</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>swe_dominant</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>sufficient</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="B15" t="inlineStr">
@@ -1410,6 +1765,31 @@
           <t>Pass</t>
         </is>
       </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>Materials Science</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>joint</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>sufficient</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="B16" t="inlineStr">
@@ -1473,6 +1853,31 @@
           <t>Pass</t>
         </is>
       </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>Materials Science</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>joint</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>sufficient</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="B17" t="inlineStr">
@@ -1536,6 +1941,31 @@
           <t>Update: add another paired issue https://github.com/lammps/lammps/issues/4398</t>
         </is>
       </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>Materials Science</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>joint</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>sufficient</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="B18" t="inlineStr">
@@ -1599,6 +2029,31 @@
           <t>Update: add another paired issue https://github.com/lammps/lammps/issues/4398</t>
         </is>
       </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>Chemistry</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>joint</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>sufficient</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="B19" t="inlineStr">
@@ -1662,6 +2117,31 @@
           <t>Update: remove #4499, add another paired issue https://github.com/lammps/lammps/issues/4491</t>
         </is>
       </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>Materials Science</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>joint</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>sufficient</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="B20" t="inlineStr">
@@ -1723,6 +2203,31 @@
       <c r="P20" t="inlineStr">
         <is>
           <t>Update: remove #4499, add another paired issue https://github.com/lammps/lammps/issues/4491</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>Materials Science</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>joint</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>sufficient</t>
         </is>
       </c>
     </row>
@@ -1795,6 +2300,31 @@
           <t>Pass</t>
         </is>
       </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>Materials Science</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>swe_dominant</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>sufficient</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="B22" t="inlineStr">
@@ -1864,6 +2394,31 @@
           <t>Pass</t>
         </is>
       </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>Physics</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>science_dominant</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>sufficient</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="B23" t="inlineStr">
@@ -1927,6 +2482,31 @@
           <t>Pass</t>
         </is>
       </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>Materials Science</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>joint</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>sufficient</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="B24" t="inlineStr">
@@ -1990,6 +2570,31 @@
           <t>Pass</t>
         </is>
       </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>Chemistry</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>swe_dominant</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>sufficient</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="B25" t="inlineStr">
@@ -2054,6 +2659,31 @@
           <t>Pass</t>
         </is>
       </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>Materials Science</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>joint</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>sufficient</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="B26" t="inlineStr">
@@ -2122,6 +2752,31 @@
           <t>Pass</t>
         </is>
       </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>Materials Science</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>joint</t>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="U26" t="inlineStr">
+        <is>
+          <t>sufficient</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="B27" t="inlineStr">
@@ -2185,6 +2840,31 @@
           <t>Pass</t>
         </is>
       </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>Materials Science</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>joint</t>
+        </is>
+      </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="U27" t="inlineStr">
+        <is>
+          <t>sufficient</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="B28" t="inlineStr">
@@ -2248,6 +2928,31 @@
           <t>Pass</t>
         </is>
       </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>Physics</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>joint</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="U28" t="inlineStr">
+        <is>
+          <t>sufficient</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2311,6 +3016,31 @@
           <t>Pass</t>
         </is>
       </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>Chemistry</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>joint</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="U29" t="inlineStr">
+        <is>
+          <t>sufficient</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2374,6 +3104,31 @@
           <t>Pass</t>
         </is>
       </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>Materials Science</t>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>joint</t>
+        </is>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="U30" t="inlineStr">
+        <is>
+          <t>sufficient</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2442,6 +3197,31 @@
           <t>Pass</t>
         </is>
       </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>Chemistry</t>
+        </is>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>joint</t>
+        </is>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="U31" t="inlineStr">
+        <is>
+          <t>sufficient</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2505,6 +3285,31 @@
           <t>Pass</t>
         </is>
       </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>Chemistry</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>swe_dominant</t>
+        </is>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>sufficient</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2568,6 +3373,31 @@
           <t>Pass</t>
         </is>
       </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>Chemistry</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>joint</t>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="U33" t="inlineStr">
+        <is>
+          <t>sufficient</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2631,6 +3461,31 @@
           <t>Pass</t>
         </is>
       </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>Materials Science</t>
+        </is>
+      </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>science_dominant</t>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="T34" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="U34" t="inlineStr">
+        <is>
+          <t>sufficient</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2699,6 +3554,31 @@
           <t>Pass</t>
         </is>
       </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>Chemistry</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>joint</t>
+        </is>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="T35" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="U35" t="inlineStr">
+        <is>
+          <t>sufficient</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2762,6 +3642,31 @@
           <t>Pass: PR rejects a type support, while both ds and gpt chose to support it, which should not be supported</t>
         </is>
       </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>Chemistry</t>
+        </is>
+      </c>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>swe_dominant</t>
+        </is>
+      </c>
+      <c r="S36" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="T36" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="U36" t="inlineStr">
+        <is>
+          <t>insufficient</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2825,6 +3730,31 @@
           <t>Pass</t>
         </is>
       </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>Chemistry</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>swe_dominant</t>
+        </is>
+      </c>
+      <c r="S37" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="T37" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="U37" t="inlineStr">
+        <is>
+          <t>sufficient</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2894,6 +3824,31 @@
           <t>Pass</t>
         </is>
       </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>Chemistry</t>
+        </is>
+      </c>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>joint</t>
+        </is>
+      </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="T38" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="U38" t="inlineStr">
+        <is>
+          <t>sufficient</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2957,6 +3912,31 @@
           <t>Pass: maintainer suggests another root cause, not the bug described in the issue</t>
         </is>
       </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>Chemistry</t>
+        </is>
+      </c>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>joint</t>
+        </is>
+      </c>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="T39" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="U39" t="inlineStr">
+        <is>
+          <t>sufficient</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -3020,6 +4000,31 @@
           <t>Pass</t>
         </is>
       </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>Chemistry</t>
+        </is>
+      </c>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>swe_dominant</t>
+        </is>
+      </c>
+      <c r="S40" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="T40" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="U40" t="inlineStr">
+        <is>
+          <t>sufficient</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -3083,6 +4088,31 @@
           <t>Pass</t>
         </is>
       </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>Chemistry</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>swe_dominant</t>
+        </is>
+      </c>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="T41" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="U41" t="inlineStr">
+        <is>
+          <t>sufficient</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -3151,6 +4181,31 @@
           <t>Pass: the root cause is not so obvious as explained in the issue description</t>
         </is>
       </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>Chemistry</t>
+        </is>
+      </c>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>swe_dominant</t>
+        </is>
+      </c>
+      <c r="S42" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="T42" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="U42" t="inlineStr">
+        <is>
+          <t>sufficient</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -3214,6 +4269,31 @@
           <t>Pass</t>
         </is>
       </c>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>Chemistry</t>
+        </is>
+      </c>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>joint</t>
+        </is>
+      </c>
+      <c r="S43" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="T43" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="U43" t="inlineStr">
+        <is>
+          <t>sufficient</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -3282,6 +4362,31 @@
           <t>Pass</t>
         </is>
       </c>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>Physics</t>
+        </is>
+      </c>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>swe_dominant</t>
+        </is>
+      </c>
+      <c r="S44" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="T44" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="U44" t="inlineStr">
+        <is>
+          <t>sufficient</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -3345,6 +4450,31 @@
           <t>Pass</t>
         </is>
       </c>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>Chemistry</t>
+        </is>
+      </c>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>swe_dominant</t>
+        </is>
+      </c>
+      <c r="S45" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="T45" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="U45" t="inlineStr">
+        <is>
+          <t>sufficient</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -3411,6 +4541,31 @@
       <c r="P46" t="inlineStr">
         <is>
           <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q46" t="inlineStr">
+        <is>
+          <t>Materials Science</t>
+        </is>
+      </c>
+      <c r="R46" t="inlineStr">
+        <is>
+          <t>joint</t>
+        </is>
+      </c>
+      <c r="S46" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="T46" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="U46" t="inlineStr">
+        <is>
+          <t>sufficient</t>
         </is>
       </c>
     </row>
@@ -3483,6 +4638,31 @@
           <t>Pass</t>
         </is>
       </c>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>Chemistry</t>
+        </is>
+      </c>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>swe_dominant</t>
+        </is>
+      </c>
+      <c r="S47" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="T47" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="U47" t="inlineStr">
+        <is>
+          <t>sufficient</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -3551,6 +4731,31 @@
           <t>Pass</t>
         </is>
       </c>
+      <c r="Q48" t="inlineStr">
+        <is>
+          <t>Chemistry</t>
+        </is>
+      </c>
+      <c r="R48" t="inlineStr">
+        <is>
+          <t>joint</t>
+        </is>
+      </c>
+      <c r="S48" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="T48" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="U48" t="inlineStr">
+        <is>
+          <t>sufficient</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -3625,6 +4830,31 @@
           <t>Pass</t>
         </is>
       </c>
+      <c r="Q49" t="inlineStr">
+        <is>
+          <t>Chemistry</t>
+        </is>
+      </c>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>swe_dominant</t>
+        </is>
+      </c>
+      <c r="S49" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="T49" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="U49" t="inlineStr">
+        <is>
+          <t>sufficient</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -3688,6 +4918,31 @@
           <t>Pass</t>
         </is>
       </c>
+      <c r="Q50" t="inlineStr">
+        <is>
+          <t>Chemistry</t>
+        </is>
+      </c>
+      <c r="R50" t="inlineStr">
+        <is>
+          <t>joint</t>
+        </is>
+      </c>
+      <c r="S50" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="T50" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="U50" t="inlineStr">
+        <is>
+          <t>sufficient</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -3751,6 +5006,31 @@
           <t>Pass</t>
         </is>
       </c>
+      <c r="Q51" t="inlineStr">
+        <is>
+          <t>Chemistry</t>
+        </is>
+      </c>
+      <c r="R51" t="inlineStr">
+        <is>
+          <t>swe_dominant</t>
+        </is>
+      </c>
+      <c r="S51" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="T51" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="U51" t="inlineStr">
+        <is>
+          <t>sufficient</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -3819,6 +5099,31 @@
           <t>Pass</t>
         </is>
       </c>
+      <c r="Q52" t="inlineStr">
+        <is>
+          <t>Chemistry</t>
+        </is>
+      </c>
+      <c r="R52" t="inlineStr">
+        <is>
+          <t>swe_dominant</t>
+        </is>
+      </c>
+      <c r="S52" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="T52" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="U52" t="inlineStr">
+        <is>
+          <t>sufficient</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -3887,6 +5192,31 @@
           <t>Pass</t>
         </is>
       </c>
+      <c r="Q53" t="inlineStr">
+        <is>
+          <t>Chemistry</t>
+        </is>
+      </c>
+      <c r="R53" t="inlineStr">
+        <is>
+          <t>swe_dominant</t>
+        </is>
+      </c>
+      <c r="S53" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="T53" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="U53" t="inlineStr">
+        <is>
+          <t>sufficient</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -3960,6 +5290,31 @@
           <t>Pass</t>
         </is>
       </c>
+      <c r="Q54" t="inlineStr">
+        <is>
+          <t>Materials Science</t>
+        </is>
+      </c>
+      <c r="R54" t="inlineStr">
+        <is>
+          <t>swe_dominant</t>
+        </is>
+      </c>
+      <c r="S54" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="T54" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="U54" t="inlineStr">
+        <is>
+          <t>insufficient</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -4023,6 +5378,31 @@
           <t>Pass</t>
         </is>
       </c>
+      <c r="Q55" t="inlineStr">
+        <is>
+          <t>Chemistry</t>
+        </is>
+      </c>
+      <c r="R55" t="inlineStr">
+        <is>
+          <t>joint</t>
+        </is>
+      </c>
+      <c r="S55" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="T55" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="U55" t="inlineStr">
+        <is>
+          <t>sufficient</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -4091,6 +5471,31 @@
           <t>Pass</t>
         </is>
       </c>
+      <c r="Q56" t="inlineStr">
+        <is>
+          <t>Chemistry</t>
+        </is>
+      </c>
+      <c r="R56" t="inlineStr">
+        <is>
+          <t>swe_dominant</t>
+        </is>
+      </c>
+      <c r="S56" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="T56" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="U56" t="inlineStr">
+        <is>
+          <t>sufficient</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -4154,6 +5559,31 @@
           <t>Pass</t>
         </is>
       </c>
+      <c r="Q57" t="inlineStr">
+        <is>
+          <t>Chemistry</t>
+        </is>
+      </c>
+      <c r="R57" t="inlineStr">
+        <is>
+          <t>joint</t>
+        </is>
+      </c>
+      <c r="S57" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="T57" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="U57" t="inlineStr">
+        <is>
+          <t>sufficient</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -4222,6 +5652,31 @@
           <t>Pass</t>
         </is>
       </c>
+      <c r="Q58" t="inlineStr">
+        <is>
+          <t>Chemistry</t>
+        </is>
+      </c>
+      <c r="R58" t="inlineStr">
+        <is>
+          <t>joint</t>
+        </is>
+      </c>
+      <c r="S58" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="T58" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="U58" t="inlineStr">
+        <is>
+          <t>sufficient</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -4290,6 +5745,31 @@
           <t>Pass</t>
         </is>
       </c>
+      <c r="Q59" t="inlineStr">
+        <is>
+          <t>Chemistry</t>
+        </is>
+      </c>
+      <c r="R59" t="inlineStr">
+        <is>
+          <t>joint</t>
+        </is>
+      </c>
+      <c r="S59" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="T59" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="U59" t="inlineStr">
+        <is>
+          <t>sufficient</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -4358,6 +5838,31 @@
           <t>Pass</t>
         </is>
       </c>
+      <c r="Q60" t="inlineStr">
+        <is>
+          <t>Chemistry</t>
+        </is>
+      </c>
+      <c r="R60" t="inlineStr">
+        <is>
+          <t>swe_dominant</t>
+        </is>
+      </c>
+      <c r="S60" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="T60" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="U60" t="inlineStr">
+        <is>
+          <t>sufficient</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -4421,6 +5926,31 @@
           <t>Pass</t>
         </is>
       </c>
+      <c r="Q61" t="inlineStr">
+        <is>
+          <t>Chemistry</t>
+        </is>
+      </c>
+      <c r="R61" t="inlineStr">
+        <is>
+          <t>joint</t>
+        </is>
+      </c>
+      <c r="S61" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="T61" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="U61" t="inlineStr">
+        <is>
+          <t>sufficient</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -4484,6 +6014,31 @@
           <t>Pass</t>
         </is>
       </c>
+      <c r="Q62" t="inlineStr">
+        <is>
+          <t>Chemistry</t>
+        </is>
+      </c>
+      <c r="R62" t="inlineStr">
+        <is>
+          <t>swe_dominant</t>
+        </is>
+      </c>
+      <c r="S62" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="T62" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="U62" t="inlineStr">
+        <is>
+          <t>sufficient</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -4547,6 +6102,31 @@
           <t>Pass</t>
         </is>
       </c>
+      <c r="Q63" t="inlineStr">
+        <is>
+          <t>Chemistry</t>
+        </is>
+      </c>
+      <c r="R63" t="inlineStr">
+        <is>
+          <t>joint</t>
+        </is>
+      </c>
+      <c r="S63" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="T63" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="U63" t="inlineStr">
+        <is>
+          <t>sufficient</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -4610,6 +6190,31 @@
           <t>Pass</t>
         </is>
       </c>
+      <c r="Q64" t="inlineStr">
+        <is>
+          <t>Chemistry</t>
+        </is>
+      </c>
+      <c r="R64" t="inlineStr">
+        <is>
+          <t>joint</t>
+        </is>
+      </c>
+      <c r="S64" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="T64" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="U64" t="inlineStr">
+        <is>
+          <t>sufficient</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -4679,6 +6284,31 @@
           <t>Pass</t>
         </is>
       </c>
+      <c r="Q65" t="inlineStr">
+        <is>
+          <t>Chemistry</t>
+        </is>
+      </c>
+      <c r="R65" t="inlineStr">
+        <is>
+          <t>joint</t>
+        </is>
+      </c>
+      <c r="S65" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="T65" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="U65" t="inlineStr">
+        <is>
+          <t>sufficient</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -4745,6 +6375,31 @@
       <c r="P66" t="inlineStr">
         <is>
           <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q66" t="inlineStr">
+        <is>
+          <t>Chemistry</t>
+        </is>
+      </c>
+      <c r="R66" t="inlineStr">
+        <is>
+          <t>joint</t>
+        </is>
+      </c>
+      <c r="S66" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="T66" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="U66" t="inlineStr">
+        <is>
+          <t>sufficient</t>
         </is>
       </c>
     </row>
@@ -4817,6 +6472,31 @@
           <t>Pass</t>
         </is>
       </c>
+      <c r="Q67" t="inlineStr">
+        <is>
+          <t>Chemistry</t>
+        </is>
+      </c>
+      <c r="R67" t="inlineStr">
+        <is>
+          <t>joint</t>
+        </is>
+      </c>
+      <c r="S67" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="T67" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="U67" t="inlineStr">
+        <is>
+          <t>sufficient</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -4880,6 +6560,31 @@
           <t>Pass</t>
         </is>
       </c>
+      <c r="Q68" t="inlineStr">
+        <is>
+          <t>Chemistry</t>
+        </is>
+      </c>
+      <c r="R68" t="inlineStr">
+        <is>
+          <t>swe_dominant</t>
+        </is>
+      </c>
+      <c r="S68" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="T68" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="U68" t="inlineStr">
+        <is>
+          <t>insufficient</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -4943,6 +6648,31 @@
           <t>Pass</t>
         </is>
       </c>
+      <c r="Q69" t="inlineStr">
+        <is>
+          <t>Chemistry</t>
+        </is>
+      </c>
+      <c r="R69" t="inlineStr">
+        <is>
+          <t>joint</t>
+        </is>
+      </c>
+      <c r="S69" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="T69" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="U69" t="inlineStr">
+        <is>
+          <t>sufficient</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -5006,6 +6736,31 @@
           <t>Pass</t>
         </is>
       </c>
+      <c r="Q70" t="inlineStr">
+        <is>
+          <t>Chemistry</t>
+        </is>
+      </c>
+      <c r="R70" t="inlineStr">
+        <is>
+          <t>swe_dominant</t>
+        </is>
+      </c>
+      <c r="S70" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="T70" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="U70" t="inlineStr">
+        <is>
+          <t>sufficient</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -5069,6 +6824,31 @@
           <t>Pass: the maintainer said it is hard to find a test</t>
         </is>
       </c>
+      <c r="Q71" t="inlineStr">
+        <is>
+          <t>Materials Science</t>
+        </is>
+      </c>
+      <c r="R71" t="inlineStr">
+        <is>
+          <t>joint</t>
+        </is>
+      </c>
+      <c r="S71" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="T71" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="U71" t="inlineStr">
+        <is>
+          <t>sufficient</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -5130,6 +6910,31 @@
       <c r="P72" t="inlineStr">
         <is>
           <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q72" t="inlineStr">
+        <is>
+          <t>Chemistry</t>
+        </is>
+      </c>
+      <c r="R72" t="inlineStr">
+        <is>
+          <t>swe_dominant</t>
+        </is>
+      </c>
+      <c r="S72" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="T72" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="U72" t="inlineStr">
+        <is>
+          <t>sufficient</t>
         </is>
       </c>
     </row>
@@ -5205,6 +7010,31 @@
           <t>Pass</t>
         </is>
       </c>
+      <c r="Q73" t="inlineStr">
+        <is>
+          <t>Chemistry</t>
+        </is>
+      </c>
+      <c r="R73" t="inlineStr">
+        <is>
+          <t>joint</t>
+        </is>
+      </c>
+      <c r="S73" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="T73" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="U73" t="inlineStr">
+        <is>
+          <t>sufficient</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -5280,6 +7110,31 @@
           <t>Pass</t>
         </is>
       </c>
+      <c r="Q74" t="inlineStr">
+        <is>
+          <t>Chemistry</t>
+        </is>
+      </c>
+      <c r="R74" t="inlineStr">
+        <is>
+          <t>science_dominant</t>
+        </is>
+      </c>
+      <c r="S74" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="T74" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="U74" t="inlineStr">
+        <is>
+          <t>sufficient</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="B75" t="inlineStr">
@@ -5343,6 +7198,31 @@
           <t>Pass</t>
         </is>
       </c>
+      <c r="Q75" t="inlineStr">
+        <is>
+          <t>Materials Science</t>
+        </is>
+      </c>
+      <c r="R75" t="inlineStr">
+        <is>
+          <t>joint</t>
+        </is>
+      </c>
+      <c r="S75" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="T75" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="U75" t="inlineStr">
+        <is>
+          <t>sufficient</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="B76" t="inlineStr">
@@ -5406,6 +7286,31 @@
           <t>Pass</t>
         </is>
       </c>
+      <c r="Q76" t="inlineStr">
+        <is>
+          <t>Materials Science</t>
+        </is>
+      </c>
+      <c r="R76" t="inlineStr">
+        <is>
+          <t>swe_dominant</t>
+        </is>
+      </c>
+      <c r="S76" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="T76" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="U76" t="inlineStr">
+        <is>
+          <t>insufficient</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="B77" t="inlineStr">
@@ -5470,6 +7375,31 @@
           <t>Pass</t>
         </is>
       </c>
+      <c r="Q77" t="inlineStr">
+        <is>
+          <t>Materials Science</t>
+        </is>
+      </c>
+      <c r="R77" t="inlineStr">
+        <is>
+          <t>joint</t>
+        </is>
+      </c>
+      <c r="S77" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="T77" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="U77" t="inlineStr">
+        <is>
+          <t>sufficient</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="B78" t="inlineStr">
@@ -5534,6 +7464,31 @@
           <t>Pass</t>
         </is>
       </c>
+      <c r="Q78" t="inlineStr">
+        <is>
+          <t>Materials Science</t>
+        </is>
+      </c>
+      <c r="R78" t="inlineStr">
+        <is>
+          <t>joint</t>
+        </is>
+      </c>
+      <c r="S78" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="T78" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="U78" t="inlineStr">
+        <is>
+          <t>sufficient</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="B79" t="inlineStr">
@@ -5598,6 +7553,31 @@
           <t>Pass</t>
         </is>
       </c>
+      <c r="Q79" t="inlineStr">
+        <is>
+          <t>Materials Science</t>
+        </is>
+      </c>
+      <c r="R79" t="inlineStr">
+        <is>
+          <t>joint</t>
+        </is>
+      </c>
+      <c r="S79" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="T79" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="U79" t="inlineStr">
+        <is>
+          <t>sufficient</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="B80" t="inlineStr">
@@ -5661,6 +7641,31 @@
           <t>Pass</t>
         </is>
       </c>
+      <c r="Q80" t="inlineStr">
+        <is>
+          <t>Materials Science</t>
+        </is>
+      </c>
+      <c r="R80" t="inlineStr">
+        <is>
+          <t>swe_dominant</t>
+        </is>
+      </c>
+      <c r="S80" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="T80" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="U80" t="inlineStr">
+        <is>
+          <t>insufficient</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="B81" t="inlineStr">
@@ -5724,6 +7729,31 @@
           <t>Update: add another two PR-paired issues https://github.com/lammps/lammps/issues/4337 and https://github.com/lammps/lammps/issues/4216</t>
         </is>
       </c>
+      <c r="Q81" t="inlineStr">
+        <is>
+          <t>Materials Science</t>
+        </is>
+      </c>
+      <c r="R81" t="inlineStr">
+        <is>
+          <t>swe_dominant</t>
+        </is>
+      </c>
+      <c r="S81" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="T81" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="U81" t="inlineStr">
+        <is>
+          <t>sufficient</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="B82" t="inlineStr">
@@ -5787,6 +7817,31 @@
           <t>Pass</t>
         </is>
       </c>
+      <c r="Q82" t="inlineStr">
+        <is>
+          <t>Materials Science</t>
+        </is>
+      </c>
+      <c r="R82" t="inlineStr">
+        <is>
+          <t>swe_dominant</t>
+        </is>
+      </c>
+      <c r="S82" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="T82" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="U82" t="inlineStr">
+        <is>
+          <t>insufficient</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="B83" t="inlineStr">
@@ -5843,6 +7898,31 @@
       <c r="P83" t="inlineStr">
         <is>
           <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q83" t="inlineStr">
+        <is>
+          <t>Bioinformatics</t>
+        </is>
+      </c>
+      <c r="R83" t="inlineStr">
+        <is>
+          <t>swe_dominant</t>
+        </is>
+      </c>
+      <c r="S83" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="T83" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="U83" t="inlineStr">
+        <is>
+          <t>insufficient</t>
         </is>
       </c>
     </row>
@@ -5910,6 +7990,31 @@
           <t>Pass</t>
         </is>
       </c>
+      <c r="Q84" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="R84" t="inlineStr">
+        <is>
+          <t>swe_dominant</t>
+        </is>
+      </c>
+      <c r="S84" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="T84" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="U84" t="inlineStr">
+        <is>
+          <t>insufficient</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="B85" t="inlineStr">
@@ -5975,6 +8080,31 @@
           <t>Pass</t>
         </is>
       </c>
+      <c r="Q85" t="inlineStr">
+        <is>
+          <t>Astronomy</t>
+        </is>
+      </c>
+      <c r="R85" t="inlineStr">
+        <is>
+          <t>swe_dominant</t>
+        </is>
+      </c>
+      <c r="S85" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="T85" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="U85" t="inlineStr">
+        <is>
+          <t>insufficient</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="B86" t="inlineStr">
@@ -6038,6 +8168,31 @@
           <t>Pass</t>
         </is>
       </c>
+      <c r="Q86" t="inlineStr">
+        <is>
+          <t>Physics</t>
+        </is>
+      </c>
+      <c r="R86" t="inlineStr">
+        <is>
+          <t>swe_dominant</t>
+        </is>
+      </c>
+      <c r="S86" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="T86" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="U86" t="inlineStr">
+        <is>
+          <t>sufficient</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="B87" t="inlineStr">
@@ -6101,6 +8256,31 @@
           <t>Pass</t>
         </is>
       </c>
+      <c r="Q87" t="inlineStr">
+        <is>
+          <t>Physics</t>
+        </is>
+      </c>
+      <c r="R87" t="inlineStr">
+        <is>
+          <t>joint</t>
+        </is>
+      </c>
+      <c r="S87" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="T87" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="U87" t="inlineStr">
+        <is>
+          <t>sufficient</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="B88" t="inlineStr">
@@ -6159,6 +8339,31 @@
           <t>Pass</t>
         </is>
       </c>
+      <c r="Q88" t="inlineStr">
+        <is>
+          <t>Chemistry</t>
+        </is>
+      </c>
+      <c r="R88" t="inlineStr">
+        <is>
+          <t>swe_dominant</t>
+        </is>
+      </c>
+      <c r="S88" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="T88" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="U88" t="inlineStr">
+        <is>
+          <t>insufficient</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="B89" t="inlineStr">
@@ -6221,6 +8426,31 @@
       <c r="P89" t="inlineStr">
         <is>
           <t>Pass</t>
+        </is>
+      </c>
+      <c r="Q89" t="inlineStr">
+        <is>
+          <t>Chemistry</t>
+        </is>
+      </c>
+      <c r="R89" t="inlineStr">
+        <is>
+          <t>swe_dominant</t>
+        </is>
+      </c>
+      <c r="S89" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="T89" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="U89" t="inlineStr">
+        <is>
+          <t>sufficient</t>
         </is>
       </c>
     </row>

</xml_diff>